<commit_message>
Complete confirmatory analysis and Nature Communications release
</commit_message>
<xml_diff>
--- a/paper/supplementary_data/Supplementary_Data_1_experiment_ledger.xlsx
+++ b/paper/supplementary_data/Supplementary_Data_1_experiment_ledger.xlsx
@@ -425,21 +425,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="60" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="37" customWidth="1" min="3" max="3"/>
-    <col width="49" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
-    <col width="27" customWidth="1" min="7" max="7"/>
-    <col width="45" customWidth="1" min="8" max="8"/>
-    <col width="21" customWidth="1" min="9" max="9"/>
-    <col width="31" customWidth="1" min="10" max="10"/>
-    <col width="23" customWidth="1" min="11" max="11"/>
-    <col width="48" customWidth="1" min="12" max="12"/>
+    <col width="58" customWidth="1" min="1" max="1"/>
+    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="58" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -455,1310 +451,868 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>physical_source</t>
+          <t>physical source</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>target</t>
+          <t>analysis ID</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>model</t>
+          <t>evaluation</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>inference_requirement</t>
+          <t>MAE (kcal/mol)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>evaluation_regime</t>
+          <t>role in final model</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>leakage_rule</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>mae_kcal_mol</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>result_interpretation</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>role_in_final_model</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>artifact_path</t>
+          <t>artifact</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Previous structure-only</t>
+          <t>Matched structure-only</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Can molecular structure alone recover hydration free energy?</t>
+          <t>Do response priors add information?</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>RDKit descriptors + Morgan</t>
+          <t>none</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>experimental hydration</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ExtraTrees</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>structure only</t>
-        </is>
+          <t>fixed five-fold OOF</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>0.3033484655954973</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>five-fold random OOF</t>
+          <t>matched control</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>molecule-disjoint outer folds</t>
-        </is>
-      </c>
-      <c r="I2" t="n">
-        <v>0.238606118980392</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>baseline</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>superseded</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>results/predictions/headline_oof.parquet</t>
+          <t>results/confirmatory/standardized_exclusion_endpoint_predictions.parquet</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Narrow response</t>
+          <t>Empirical/residual block</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Do compact solvation-response coordinates improve the endpoint?</t>
+          <t>Do compact empirical axes and corrected responses help?</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CombiSolv-QM, Abraham, OpenFF, GBn2</t>
+          <t>Abraham, OpenFF, GBn2</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>response priors + experimental hydration</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>surrogate stack + ExtraTrees</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>structure only</t>
-        </is>
+          <t>fixed five-fold OOF</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>0.2427114968435518</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>five-fold random OOF</t>
+          <t>component</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>external benchmark connectivity removed</t>
-        </is>
-      </c>
-      <c r="I3" t="n">
-        <v>0.2136151731870528</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>improved</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>final-model component</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>results/predictions/headline_oof.parquet</t>
+          <t>results/confirmatory/standardized_exclusion_endpoint_predictions.parquet</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SMD-water response</t>
+          <t>Computation core</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Does aligned water response close the remaining gap?</t>
+          <t>Do raw computed responses help?</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>MolSolv SMD(water)</t>
+          <t>CombiSolv-QM, OpenFF, GBn2</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>SMD response + experimental hydration</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>D-MPNN surrogate + ExtraTrees</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>structure only</t>
-        </is>
+          <t>fixed five-fold OOF</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>0.2526797708683475</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>five-fold random OOF</t>
+          <t>component</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>85 benchmark connectivities removed</t>
-        </is>
-      </c>
-      <c r="I4" t="n">
-        <v>0.2016070042016807</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>improved</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>final-model component</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>results/predictions/headline_oof.parquet</t>
+          <t>results/confirmatory/standardized_exclusion_endpoint_predictions.parquet</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ConfSolv response hierarchy</t>
+          <t>SMD water</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Does conformational solvent response add transferable information?</t>
+          <t>Does water-specific continuum response transfer?</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ConfSolv H2O</t>
+          <t>MolSolv SMD</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>six response summaries + experimental hydration</t>
+          <t>D</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>LightGBM surrogates + ExtraTrees</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>structure only</t>
-        </is>
+          <t>fixed five-fold OOF</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>0.2531149568445899</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>five-fold random OOF</t>
+          <t>component</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>13 benchmark connectivities removed</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>0.1970474740948231</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>best fixed point estimate</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>final-model component</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>results/predictions/headline_oof.parquet</t>
+          <t>results/confirmatory/standardized_exclusion_endpoint_predictions.parquet</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Nested feature-block selection</t>
+          <t>ConfSolv</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Does feature-block selection preserve the result when nested?</t>
+          <t>Do conformational response summaries transfer?</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>all retained response blocks</t>
+          <t>ConfSolv H2O</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>experimental hydration</t>
+          <t>E</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>nested ExtraTrees</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>structure only</t>
-        </is>
+          <t>fixed five-fold OOF</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>0.2989909179660747</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>nested five-fold OOF</t>
+          <t>component</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>selection restricted to outer training data</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>0.1993060393064633</v>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>PIMD8-level point estimate</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>evaluation only</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>results/predictions/headline_oof.parquet</t>
+          <t>results/confirmatory/standardized_exclusion_endpoint_predictions.parquet</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Family holdout</t>
+          <t>Full SolvAI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>How does SolvAI transfer to an unseen functional family?</t>
+          <t>Do aligned response priors improve the matched endpoint?</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>final SolvAI</t>
+          <t>15 priors</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>experimental hydration</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>frozen stack</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>structure only</t>
-        </is>
+          <t>fixed five-fold OOF</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>0.2022340672191099</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>GroupKFold family holdout</t>
+          <t>final model</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>families confined to one outer fold</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>0.2395665848765438</v>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>harder chemical extrapolation</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>evaluation only</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>results/predictions/hard_holdout_oof.parquet</t>
+          <t>results/confirmatory/standardized_exclusion_endpoint_predictions.parquet</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Scaffold holdout</t>
+          <t>Shuffled priors</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>How does SolvAI transfer to unseen scaffolds?</t>
+          <t>Does molecule-response alignment matter?</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>final SolvAI</t>
+          <t>15 permuted priors</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>experimental hydration</t>
+          <t>negative control</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>frozen stack</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>structure only</t>
-        </is>
-      </c>
+          <t>five permutations × six partitions</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>scaffold holdout</t>
+          <t>evaluation only</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>scaffolds confined to one outer fold</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
-        <v>0.2412820403309476</v>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>harder chemical extrapolation</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>evaluation only</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>results/predictions/hard_holdout_oof.parquet</t>
+          <t>results/confirmatory/standardized_exclusion_endpoint_shuffle_predictions.parquet</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>matched one seed base</t>
+          <t>Zero-ARROW transfer</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Can this alternative physical representation improve transfer?</t>
+          <t>Do priors help without ARROW endpoint labels?</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>matched_one_seed_base</t>
+          <t>15 priors</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>experimental hydration</t>
+          <t>transfer control</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>documented frozen screen</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>structure only</t>
-        </is>
+          <t>all 85 as test</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>0.2569405918663764</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>matched OOF screen</t>
+          <t>evaluation only</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>benchmark labels absent from held-out fit</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
-        <v>0.1919131084189228</v>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>non-improving screen</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>not retained</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>results/ablations/matched_one_seed_base.csv</t>
+          <t>results/confirmatory/standardized_exclusion_endpoint_predictions.parquet</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>openfe diagnostics</t>
+          <t>global_butina_0_70</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Can this alternative physical representation improve transfer?</t>
+          <t>Does the prior advantage survive global chemical separation?</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>openfe_diagnostics</t>
+          <t>15 priors</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>experimental hydration</t>
+          <t>separation control</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>documented frozen screen</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>structure only</t>
-        </is>
+          <t>global_butina_0_70</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>0.2157005113160082</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>matched OOF screen</t>
+          <t>evaluation only</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>benchmark labels absent from held-out fit</t>
-        </is>
-      </c>
-      <c r="I10" t="n">
-        <v>0.2057451966230934</v>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>non-improving screen</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>not retained</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>results/ablations/openfe_diagnostics.csv</t>
+          <t>results/confirmatory/standardized_exclusion_global_separation_predictions.parquet</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>mlff hierarchy</t>
+          <t>global_family</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Can this alternative physical representation improve transfer?</t>
+          <t>Does the prior advantage survive global chemical separation?</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>mlff_hierarchy</t>
+          <t>15 priors</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>experimental hydration</t>
+          <t>separation control</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>documented frozen screen</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>structure only</t>
-        </is>
+          <t>global_family</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>0.4677933152583255</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>matched OOF screen</t>
+          <t>evaluation only</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>benchmark labels absent from held-out fit</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
-        <v>0.2010876031746034</v>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>non-improving screen</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>not retained</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>results/ablations/mlff_hierarchy.csv</t>
+          <t>results/confirmatory/standardized_exclusion_global_separation_predictions.parquet</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>des370k water response</t>
+          <t>global_nn_0.50</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Can this alternative physical representation improve transfer?</t>
+          <t>Does the prior advantage survive global chemical separation?</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>des370k_water_response</t>
+          <t>15 priors</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>experimental hydration</t>
+          <t>separation control</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>documented frozen screen</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>structure only</t>
-        </is>
+          <t>global_nn_0.50</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>0.2186971786544248</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>matched OOF screen</t>
+          <t>evaluation only</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>benchmark labels absent from held-out fit</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
-        <v>0.2099278784936193</v>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>non-improving screen</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>not retained</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>results/ablations/des370k_water_response.csv</t>
+          <t>results/confirmatory/standardized_exclusion_global_separation_predictions.parquet</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>qmpff typed structure</t>
+          <t>global_nn_0.60</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Can this alternative physical representation improve transfer?</t>
+          <t>Does the prior advantage survive global chemical separation?</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>qmpff_typed_structure</t>
+          <t>15 priors</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>experimental hydration</t>
+          <t>separation control</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>documented frozen screen</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>structure only</t>
-        </is>
+          <t>global_nn_0.60</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>0.2113965726138604</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>matched OOF screen</t>
+          <t>evaluation only</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>benchmark labels absent from held-out fit</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>0.2088045993230627</v>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>non-improving screen</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>not retained</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>results/ablations/qmpff_typed_structure.csv</t>
+          <t>results/confirmatory/standardized_exclusion_global_separation_predictions.parquet</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>gnnis force response</t>
+          <t>global_nn_0.70</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Can this alternative physical representation improve transfer?</t>
+          <t>Does the prior advantage survive global chemical separation?</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>gnnis_force_response</t>
+          <t>15 priors</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>experimental hydration</t>
+          <t>separation control</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>documented frozen screen</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>structure only</t>
-        </is>
+          <t>global_nn_0.70</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>0.2109972548760245</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>matched OOF screen</t>
+          <t>evaluation only</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>benchmark labels absent from held-out fit</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>0.207935233426704</v>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>non-improving screen</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>not retained</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>results/ablations/gnnis_force_response.csv</t>
+          <t>results/confirmatory/standardized_exclusion_global_separation_predictions.parquet</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>lambda aware implicit</t>
+          <t>global_nn_0.80</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Can this alternative physical representation improve transfer?</t>
+          <t>Does the prior advantage survive global chemical separation?</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>lambda_aware_implicit</t>
+          <t>15 priors</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>experimental hydration</t>
+          <t>separation control</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>documented frozen screen</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>structure only</t>
-        </is>
+          <t>global_nn_0.80</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>0.209515344203237</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>matched OOF screen</t>
+          <t>evaluation only</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>benchmark labels absent from held-out fit</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
-        <v>0.2097411174291937</v>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>non-improving screen</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>not retained</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>results/ablations/lambda_aware_implicit.csv</t>
+          <t>results/confirmatory/standardized_exclusion_global_separation_predictions.parquet</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>phase space dynamic</t>
+          <t>global_scaffold</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Can this alternative physical representation improve transfer?</t>
+          <t>Does the prior advantage survive global chemical separation?</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>phase_space_dynamic</t>
+          <t>15 priors</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>experimental hydration</t>
+          <t>separation control</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>documented frozen screen</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>structure only</t>
-        </is>
+          <t>global_scaffold</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>0.3761935493360304</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>matched OOF screen</t>
+          <t>evaluation only</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>benchmark labels absent from held-out fit</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
-        <v>0.2189401242880484</v>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>non-improving screen</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>not retained</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>results/ablations/phase_space_dynamic.csv</t>
+          <t>results/confirmatory/standardized_exclusion_global_separation_predictions.parquet</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>gnequip hierarchy</t>
+          <t>matched one seed base</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Can this alternative physical representation improve transfer?</t>
+          <t>Can an alternative physical representation improve transfer?</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>gnequip_hierarchy</t>
+          <t>matched_one_seed_base</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>experimental hydration</t>
+          <t>exploratory</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>documented frozen screen</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>structure only</t>
-        </is>
+          <t>campaign OOF screen</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>0.1919131084189228</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>matched OOF screen</t>
+          <t>not retained</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>benchmark labels absent from held-out fit</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>0.2227629413748834</v>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>non-improving screen</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>not retained</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>results/ablations/gnequip_hierarchy.csv</t>
+          <t>results/ablations/</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>confsolv graph embedding</t>
+          <t>openfe diagnostics</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Can this alternative physical representation improve transfer?</t>
+          <t>Can an alternative physical representation improve transfer?</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>confsolv_graph_embedding</t>
+          <t>openfe_diagnostics</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>experimental hydration</t>
+          <t>exploratory</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>documented frozen screen</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>structure only</t>
-        </is>
+          <t>campaign OOF screen</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>0.2057451966230934</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>matched OOF screen</t>
+          <t>not retained</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>benchmark labels absent from held-out fit</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>0.2121932664332402</v>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>non-improving screen</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>not retained</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>results/ablations/confsolv_graph_embedding.csv</t>
+          <t>results/ablations/</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>confsolv ffn embedding</t>
+          <t>mlff hierarchy</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Can this alternative physical representation improve transfer?</t>
+          <t>Can an alternative physical representation improve transfer?</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>confsolv_ffn_embedding</t>
+          <t>mlff_hierarchy</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>experimental hydration</t>
+          <t>exploratory</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>documented frozen screen</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>structure only</t>
-        </is>
+          <t>campaign OOF screen</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>0.2010876031746034</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>matched OOF screen</t>
+          <t>not retained</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>benchmark labels absent from held-out fit</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>0.2154807450202304</v>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>non-improving screen</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>not retained</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>results/ablations/confsolv_ffn_embedding.csv</t>
+          <t>results/ablations/</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>openfe nqe dpnn</t>
+          <t>des370k water response</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Can this alternative physical representation improve transfer?</t>
+          <t>Can an alternative physical representation improve transfer?</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>openfe_nqe_dpnn</t>
+          <t>des370k_water_response</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>experimental hydration</t>
+          <t>exploratory</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>documented frozen screen</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>structure only</t>
-        </is>
+          <t>campaign OOF screen</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>0.2099278784936193</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>matched OOF screen</t>
+          <t>not retained</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>benchmark labels absent from held-out fit</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>0.4750677222352941</v>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>non-improving screen</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>not retained</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>results/ablations/openfe_nqe_dpnn.csv</t>
+          <t>results/ablations/</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>molpile dpnn</t>
+          <t>Multi-lambda physics distillation A: structure/response baseline</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Can this alternative physical representation improve transfer?</t>
+          <t>Can predicted lambda response improve the endpoint?</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>molpile_dpnn</t>
+          <t>PIMD2 response</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>experimental hydration</t>
+          <t>exploratory</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>documented frozen screen</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>structure only</t>
-        </is>
+          <t>matched OOF</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>0.1959185120707542</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>matched OOF screen</t>
+          <t>not retained</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>benchmark labels absent from held-out fit</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>0.4725549945882352</v>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>non-improving screen</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>not retained</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>results/ablations/molpile_dpnn.csv</t>
+          <t>results/ablations/multilambda_metrics.csv</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Multi-lambda physics distillation A: structure/response baseline</t>
+          <t>Multi-lambda physics distillation B2: +distilled PIMD2 lambda response</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Can structure-derived lambda response improve the endpoint?</t>
+          <t>Can predicted lambda response improve the endpoint?</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>short PIMD2 lambda response</t>
+          <t>PIMD2 response</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>response hierarchy or integrated free energy</t>
+          <t>exploratory</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>masked multi-task student</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>structure only</t>
-        </is>
+          <t>matched OOF</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>0.2013553142753398</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>matched random OOF</t>
+          <t>not retained</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
-        <is>
-          <t>held-out response labels absent</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>0.1959185120707542</v>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>response-surrogate bottleneck</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>not retained</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
         <is>
           <t>results/ablations/multilambda_metrics.csv</t>
         </is>
@@ -1767,58 +1321,38 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Multi-lambda physics distillation B2: +distilled PIMD2 lambda response</t>
+          <t>Multi-lambda physics distillation B1: +distilled classical-NQE-PIMD hierarchy</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Can structure-derived lambda response improve the endpoint?</t>
+          <t>Can predicted lambda response improve the endpoint?</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>short PIMD2 lambda response</t>
+          <t>PIMD2 response</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>response hierarchy or integrated free energy</t>
+          <t>exploratory</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>masked multi-task student</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>structure only</t>
-        </is>
+          <t>matched OOF</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>0.2147409688945948</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>matched random OOF</t>
+          <t>not retained</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
-        <is>
-          <t>held-out response labels absent</t>
-        </is>
-      </c>
-      <c r="I23" t="n">
-        <v>0.2013553142753398</v>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>response-surrogate bottleneck</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>not retained</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
         <is>
           <t>results/ablations/multilambda_metrics.csv</t>
         </is>
@@ -1827,58 +1361,38 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Multi-lambda physics distillation B1: +distilled classical-NQE-PIMD hierarchy</t>
+          <t>Multi-lambda physics distillation B: +full distilled physics hierarchy</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Can structure-derived lambda response improve the endpoint?</t>
+          <t>Can predicted lambda response improve the endpoint?</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>short PIMD2 lambda response</t>
+          <t>PIMD2 response</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>response hierarchy or integrated free energy</t>
+          <t>exploratory</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>masked multi-task student</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>structure only</t>
-        </is>
+          <t>matched OOF</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>0.2190051043287684</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>matched random OOF</t>
+          <t>not retained</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
-        <is>
-          <t>held-out response labels absent</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
-        <v>0.2147409688945948</v>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>response-surrogate bottleneck</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>not retained</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
         <is>
           <t>results/ablations/multilambda_metrics.csv</t>
         </is>
@@ -1887,118 +1401,38 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Multi-lambda physics distillation B: +full distilled physics hierarchy</t>
+          <t>Multi-lambda physics distillation C: integrated predicted dH/dlambda (affine calibration)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Can structure-derived lambda response improve the endpoint?</t>
+          <t>Can predicted lambda response improve the endpoint?</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>short PIMD2 lambda response</t>
+          <t>PIMD2 response</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>response hierarchy or integrated free energy</t>
+          <t>exploratory</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>masked multi-task student</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>structure only</t>
-        </is>
+          <t>matched OOF</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>1.513562887346043</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>matched random OOF</t>
+          <t>not retained</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
-        <is>
-          <t>held-out response labels absent</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>0.2190051043287684</v>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>response-surrogate bottleneck</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>not retained</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>results/ablations/multilambda_metrics.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Multi-lambda physics distillation C: integrated predicted dH/dlambda (affine calibration)</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Can structure-derived lambda response improve the endpoint?</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>short PIMD2 lambda response</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>response hierarchy or integrated free energy</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>masked multi-task student</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>structure only</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>matched random OOF</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>held-out response labels absent</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>1.513562887346043</v>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>response-surrogate bottleneck</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>not retained</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr">
         <is>
           <t>results/ablations/multilambda_metrics.csv</t>
         </is>

</xml_diff>

<commit_message>
complete external validation and submission QA
</commit_message>
<xml_diff>
--- a/paper/supplementary_data/Supplementary_Data_1_experiment_ledger.xlsx
+++ b/paper/supplementary_data/Supplementary_Data_1_experiment_ledger.xlsx
@@ -425,14 +425,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
     <col width="58" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="33" customWidth="1" min="4" max="4"/>
+    <col width="37" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="58" customWidth="1" min="8" max="8"/>
@@ -801,12 +801,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>global_butina_0_70</t>
+          <t>ARROW weight-one sensitivity</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Does the prior advantage survive global chemical separation?</t>
+          <t>Does the response advantage depend on threefold weighting of ARROW training rows?</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -816,16 +816,16 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>separation control</t>
+          <t>prospective sensitivity</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>global_butina_0_70</t>
+          <t>fixed five-fold OOF; ARROW weight 1</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.2157005113160082</v>
+        <v>0.2064174945533771</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -834,19 +834,19 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>results/confirmatory/standardized_exclusion_global_separation_predictions.parquet</t>
+          <t>results/michael_30aug_sensitivity/weight1_predictions.parquet</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>global_family</t>
+          <t>Tier-A endpoint-disjoint external cohort</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Does the prior advantage survive global chemical separation?</t>
+          <t>Does the matched response advantage transfer beyond ARROW-85?</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -856,16 +856,16 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>separation control</t>
+          <t>prospective external validation</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>global_family</t>
+          <t>external endpoint-disjoint; n=220</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>0.4677933152583255</v>
+        <v>1.152554228782572</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -874,19 +874,19 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>results/confirmatory/standardized_exclusion_global_separation_predictions.parquet</t>
+          <t>results/tier_a_external/evaluation/tier_a_external_predictions.parquet</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>global_nn_0.50</t>
+          <t>Tier-A strict response-source-disjoint subset</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Does the prior advantage survive global chemical separation?</t>
+          <t>Does the matched response advantage survive removal of teacher-source identities?</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -896,16 +896,16 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>separation control</t>
+          <t>prospective external validation</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>global_nn_0.50</t>
+          <t>external source-disjoint; n=97</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.2186971786544248</v>
+        <v>1.535595197705888</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -914,14 +914,14 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>results/confirmatory/standardized_exclusion_global_separation_predictions.parquet</t>
+          <t>results/tier_a_external/evaluation/tier_a_external_predictions.parquet</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>global_nn_0.60</t>
+          <t>global_butina_0_70</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -941,11 +941,11 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>global_nn_0.60</t>
+          <t>global_butina_0_70</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0.2113965726138604</v>
+        <v>0.2157005113160082</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -961,7 +961,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>global_nn_0.70</t>
+          <t>global_family</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -981,11 +981,11 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>global_nn_0.70</t>
+          <t>global_family</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0.2109972548760245</v>
+        <v>0.4677933152583255</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1001,7 +1001,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>global_nn_0.80</t>
+          <t>global_nn_0.50</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1021,11 +1021,11 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>global_nn_0.80</t>
+          <t>global_nn_0.50</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.209515344203237</v>
+        <v>0.2186971786544248</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1041,7 +1041,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>global_scaffold</t>
+          <t>global_nn_0.60</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1061,11 +1061,11 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>global_scaffold</t>
+          <t>global_nn_0.60</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.3761935493360304</v>
+        <v>0.2113965726138604</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1081,127 +1081,127 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>matched one seed base</t>
+          <t>global_nn_0.70</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Can an alternative physical representation improve transfer?</t>
+          <t>Does the prior advantage survive global chemical separation?</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>matched_one_seed_base</t>
+          <t>15 priors</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>exploratory</t>
+          <t>separation control</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>campaign OOF screen</t>
+          <t>global_nn_0.70</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0.1919131084189228</v>
+        <v>0.2109972548760245</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>not retained</t>
+          <t>evaluation only</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>results/ablations/</t>
+          <t>results/confirmatory/standardized_exclusion_global_separation_predictions.parquet</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>openfe diagnostics</t>
+          <t>global_nn_0.80</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Can an alternative physical representation improve transfer?</t>
+          <t>Does the prior advantage survive global chemical separation?</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>openfe_diagnostics</t>
+          <t>15 priors</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>exploratory</t>
+          <t>separation control</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>campaign OOF screen</t>
+          <t>global_nn_0.80</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0.2057451966230934</v>
+        <v>0.209515344203237</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>not retained</t>
+          <t>evaluation only</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>results/ablations/</t>
+          <t>results/confirmatory/standardized_exclusion_global_separation_predictions.parquet</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>mlff hierarchy</t>
+          <t>global_scaffold</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Can an alternative physical representation improve transfer?</t>
+          <t>Does the prior advantage survive global chemical separation?</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>mlff_hierarchy</t>
+          <t>15 priors</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>exploratory</t>
+          <t>separation control</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>campaign OOF screen</t>
+          <t>global_scaffold</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>0.2010876031746034</v>
+        <v>0.3761935493360304</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>not retained</t>
+          <t>evaluation only</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>results/ablations/</t>
+          <t>results/confirmatory/standardized_exclusion_global_separation_predictions.parquet</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>des370k water response</t>
+          <t>matched one seed base</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1211,7 +1211,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>des370k_water_response</t>
+          <t>matched_one_seed_base</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1225,7 +1225,7 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>0.2099278784936193</v>
+        <v>0.1919131084189228</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1241,17 +1241,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Multi-lambda physics distillation A: structure/response baseline</t>
+          <t>openfe diagnostics</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Can predicted lambda response improve the endpoint?</t>
+          <t>Can an alternative physical representation improve transfer?</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>PIMD2 response</t>
+          <t>openfe_diagnostics</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1261,11 +1261,11 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>matched OOF</t>
+          <t>campaign OOF screen</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>0.1959185120707542</v>
+        <v>0.2057451966230934</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1274,24 +1274,24 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>results/ablations/multilambda_metrics.csv</t>
+          <t>results/ablations/</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Multi-lambda physics distillation B2: +distilled PIMD2 lambda response</t>
+          <t>mlff hierarchy</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Can predicted lambda response improve the endpoint?</t>
+          <t>Can an alternative physical representation improve transfer?</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>PIMD2 response</t>
+          <t>mlff_hierarchy</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1301,11 +1301,11 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>matched OOF</t>
+          <t>campaign OOF screen</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>0.2013553142753398</v>
+        <v>0.2010876031746034</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1314,24 +1314,24 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>results/ablations/multilambda_metrics.csv</t>
+          <t>results/ablations/</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Multi-lambda physics distillation B1: +distilled classical-NQE-PIMD hierarchy</t>
+          <t>des370k water response</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Can predicted lambda response improve the endpoint?</t>
+          <t>Can an alternative physical representation improve transfer?</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>PIMD2 response</t>
+          <t>des370k_water_response</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1341,11 +1341,11 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>matched OOF</t>
+          <t>campaign OOF screen</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>0.2147409688945948</v>
+        <v>0.2099278784936193</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1354,14 +1354,14 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>results/ablations/multilambda_metrics.csv</t>
+          <t>results/ablations/</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Multi-lambda physics distillation B: +full distilled physics hierarchy</t>
+          <t>Multi-lambda physics distillation A: structure/response baseline</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1385,7 +1385,7 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>0.2190051043287684</v>
+        <v>0.1959185120707542</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -1401,38 +1401,158 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>Multi-lambda physics distillation B2: +distilled PIMD2 lambda response</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Can predicted lambda response improve the endpoint?</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>PIMD2 response</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>exploratory</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>matched OOF</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>0.2013553142753398</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>not retained</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>results/ablations/multilambda_metrics.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Multi-lambda physics distillation B1: +distilled classical-NQE-PIMD hierarchy</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Can predicted lambda response improve the endpoint?</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>PIMD2 response</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>exploratory</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>matched OOF</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>0.2147409688945948</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>not retained</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>results/ablations/multilambda_metrics.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Multi-lambda physics distillation B: +full distilled physics hierarchy</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Can predicted lambda response improve the endpoint?</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>PIMD2 response</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>exploratory</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>matched OOF</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>0.2190051043287684</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>not retained</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>results/ablations/multilambda_metrics.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>Multi-lambda physics distillation C: integrated predicted dH/dlambda (affine calibration)</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>Can predicted lambda response improve the endpoint?</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>PIMD2 response</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>exploratory</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>matched OOF</t>
         </is>
       </c>
-      <c r="F25" t="n">
+      <c r="F28" t="n">
         <v>1.513562887346043</v>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>not retained</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="H28" t="inlineStr">
         <is>
           <t>results/ablations/multilambda_metrics.csv</t>
         </is>

</xml_diff>